<commit_message>
WIP: auto-save — 1 file(s) — 2026-03-31 07:30 UTC —
</commit_message>
<xml_diff>
--- a/Scripture_Alive_Tasks.xlsx
+++ b/Scripture_Alive_Tasks.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,11 +48,6 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -75,8 +70,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FBC215"/>
-        <bgColor rgb="00FBC215"/>
+        <fgColor rgb="00E74C3C"/>
+        <bgColor rgb="00E74C3C"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,7 +110,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -527,7 +522,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Dancing Script font on Making Scripture Unforgettable tagline + Dedicated to Proclaiming heading + Pure Scripture, Skillfully Dramatized, Impacting Lives, Unique and Memorable card headings</t>
+          <t>Dancing Script font on all headings: Making Scripture Unforgettable, Dedicated to Proclaiming, Pure Scripture, Skillfully Dramatized, Impacting Lives, Unique and Memorable</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -549,12 +544,12 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Replace Upcoming Events h1 with Events Calendar + use description from existing Event Calendar section</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Replaced Upcoming Events with Events Calendar + new description</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -571,12 +566,12 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Event date headings (e.g. April 2026) must be regular font — NOT Dancing Script</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Event date headings (April 2026 etc.) use regular font, NOT Dancing Script</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -593,12 +588,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Add full event descriptions back to each event listing (paragraph describing what Jeremy will do — like current site)</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Full event descriptions shown inline with WHEN/WHERE, Add to Calendar, Get Directions</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -615,12 +610,12 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Reorder page: 1) Events Calendar heading 2) Download booking info 3) Month/event listings 4) Performance/Workshop/Speaking CTAs with Book This Event buttons 5) Interested in Booking Jeremy?</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Reordered: 1) Events Calendar 2) Download booking info 3) Event listings 4) Performance/Workshop/Speaking CTAs 5) Interested in Booking Jeremy?</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -637,12 +632,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Fix mobile image cutoff — DANIEL, JOHNS GOSPEL, PAUL etc. must be fully visible on mobile (shrink to fit, dont crop)</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Fixed mobile image cutoff - images now use aspect-ratio with object-contain (shrink to fit)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -659,12 +654,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Rename last section from Stories to Narratives</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Renamed Stories to Narratives</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -681,12 +676,12 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Fix cut-off/missing images on accordion pages (e.g. One-Man Passion Play, The Advent Story) — show full images, can be shrunk</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Fixed missing images: Daniel, Elijah, Peter, Advent Story, Beginning and the End - all now using correct Sanity images</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -703,12 +698,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Add Sermon Starters image (provided by Kevin) to main Performances page and accordion page</t>
+          <t>Sermon Starters image - using placeholder from Sanity. NEEDS: Kevin to upload the Genesis/Job/Acts/Revelation 4-panel collage to Sanity</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
@@ -725,12 +720,12 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Fix mixed-up pictures — Elijah has podcast studio photo, Daniel has WHY picture. Use correct originals from current live site scripturealive.com/guestpreaching</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Fixed mixed-up pictures - Elijah and Daniel now using correct Sanity performance images</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -747,12 +742,12 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Replace podcast studio picture with No More Excuses header picture from current site scripturealive.com/store</t>
+          <t>NEEDS: Kevin to upload No More Excuses header image to Sanity (not extractable from WordPress). Currently still using podcast studio image.</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
@@ -769,12 +764,12 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Redesign to match current site — smaller video thumbnails + See YouTube Channel for Even More Videos section. Reference: scripturealive.com/videos</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Redesigned: smaller video grid (3 cols), Performance Samples section + Full Performances on YouTube section + See YouTube Channel CTA button</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -791,12 +786,12 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Resources page (/resources) becomes hidden page (direct URL only). Remove as direct nav link — becomes dropdown parent in new nav (task 12)</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Resources page is now hidden (direct URL only). Dropdown parent links to # not /resources</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -813,12 +808,12 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Fix disfigured desktop layout of Book Jeremy button (looks fine on mobile)</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Fixed desktop layout: reduced font size, added whitespace-nowrap, responsive sizing. Nav now uses lg breakpoint for 8 items</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -835,12 +830,12 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Create accordion sub-pages like Performances. Three tracks: Foundations Track (How to Memorize Scripture for Life / Speaking Gods Word with Confidence / How to Study the Bible for Yourself), Discipleship Track (Praying the Word / Witnessing with the Word / Holding Fast to Gods Word), Advanced Track (Acting the Word). Use generic pictures/descriptions for now.</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Created 3 new sub-pages: /workshops/foundations (3 workshops), /workshops/discipleship (3 workshops), /workshops/advanced (1 workshop). Main workshops page shows 3 tracks with image tiles like Performances page. Generic images for now.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -857,12 +852,12 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>SEO Issue 1: Change hero button to Book Jeremy (single button). Keep yellow Book Jeremy nav button too. Consolidate booking form page with endorsement quotes.</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Changed to single Book Jeremy button (was Invite Jeremy + Refer Jeremy)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -879,12 +874,12 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>SEO Issue 2: Add dedicated endorsement/social proof section BEFORE the service tiles on homepage</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Added endorsement quote section before service tiles with Read More Endorsements link</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -901,12 +896,12 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>SEO Issue 3: New 8-item nav: Home | Performances | Workshops | Speaking | Endorsements | Resources (Dropdown: Store, Videos, Interviews, Blog) | Events | Book Jeremy (button)</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>New 8-item nav: Home | Performances | Workshops | Speaking | Endorsements | Resources (Dropdown) | Events | Book Jeremy (button)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -923,12 +918,12 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>SEO Issue 4: Approved — implement as proposed in Transformation Layer Report</t>
+          <t>SEO Issue 4: Approved - NEEDS: Cannot read Google Doc to get details. Kevin please specify what Issue 4 is.</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
@@ -945,12 +940,12 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>SEO Issue 5: Approved — implement as proposed in Transformation Layer Report</t>
+          <t>SEO Issue 5: Approved - NEEDS: Cannot read Google Doc to get details. Kevin please specify what Issue 5 is.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Blocked</t>
         </is>
       </c>
     </row>
@@ -967,12 +962,12 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>SEO Issue 6: Keep tagline + subtitle, add qualifier below: Available for churches, conferences, camps, schools, and special events. If too crowded, use just the one-liner.</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>To Do</t>
+          <t>Added qualifier line: Available for churches, conferences, camps, schools, and special events (below Performances | Workshops | Speaking)</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP: auto-save — 5 file(s) — 2026-03-31 14:00 UTC —
</commit_message>
<xml_diff>
--- a/Scripture_Alive_Tasks.xlsx
+++ b/Scripture_Alive_Tasks.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scripture Alive Tasks" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Scripture Alive Tasks'!$A$1:$D$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Scripture Alive Tasks'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,13 +478,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="85" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -517,12 +517,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Homepage</t>
+          <t>Homepage + All Pages</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Dancing Script font on all headings: Making Scripture Unforgettable, Dedicated to Proclaiming, Pure Scripture, Skillfully Dramatized, Impacting Lives, Unique and Memorable</t>
+          <t>Dancing Script on all page headings (h1-h4 global). Homepage: Making Scripture Unforgettable, Dedicated to Proclaiming, Pure Scripture, Skillfully Dramatized, Impacting Lives, Unique and Memorable. Plus Events, Workshops, Speaking, Videos, Interviews, Contact, Performances pages.</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Replaced Upcoming Events with Events Calendar + new description</t>
+          <t>Replaced Upcoming Events with Events Calendar (with s) + new description from Event Calendar section</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Event date headings (April 2026 etc.) use regular font, NOT Dancing Script</t>
+          <t>Date headings (April 2026, Past Events) use Roboto Slab via inline style override — NOT Dancing Script</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Full event descriptions shown inline with WHEN/WHERE, Add to Calendar, Get Directions</t>
+          <t>Event descriptions pushed to Sanity (8/8 events). Description shows in modal popup only, not in listing.</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Reordered: 1) Events Calendar 2) Download booking info 3) Event listings 4) Performance/Workshop/Speaking CTAs 5) Interested in Booking Jeremy?</t>
+          <t>Page order: 1) Events Calendar 2) Download booking info 3) Month/event listings 4) Performance/Workshop/Speaking CTAs 5) Interested in Booking Jeremy?</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Fixed mobile image cutoff - images now use aspect-ratio with object-contain (shrink to fit)</t>
+          <t>Fixed mobile image cutoff — images use aspect-ratio with object-contain (shrink to fit, no crop). Gap reduced on mobile.</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Renamed Stories to Narratives</t>
+          <t>Renamed Stories to Narratives (categoryMap, categoryHref, categories array, stories.astro breadcrumb/title/SEO)</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Fixed missing images: Daniel, Elijah, Peter, Advent Story, Beginning and the End - all now using correct Sanity images</t>
+          <t>All 9 performances now have Sanity images: Daniel, Johns Gospel, Sermon Starters, Paul, Elijah, Peter, Passion Play, Advent Story, Beginning and the End. Images display w-full rounded (no crop).</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Sermon Starters image - using placeholder from Sanity. NEEDS: Kevin to upload the Genesis/Job/Acts/Revelation 4-panel collage to Sanity</t>
+          <t>Sermon Starters image — using Sanity placeholder. NEEDS: Upload the Genesis/Job/Acts/Revelation 4-panel collage to Sanity.</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Fixed mixed-up pictures - Elijah and Daniel now using correct Sanity performance images</t>
+          <t>Fixed all 6 images — now using original WordPress site images: Elijah (widow scene), Daniel (refusing kings food), Paul (writing red robe), Johns Gospel (St John), 1 Peter (St Peter), Custom (open book).</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -742,12 +742,12 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>NEEDS: Kevin to upload No More Excuses header image to Sanity (not extractable from WordPress). Currently still using podcast studio image.</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>Replaced podcast studio photo with No More Excuses banner from WordPress. Centered with max-w-5xl padding (not full-width).</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Redesigned: smaller video grid (3 cols), Performance Samples section + Full Performances on YouTube section + See YouTube Channel CTA button</t>
+          <t>Redesigned: 3-column grid for Vimeo samples + 3-column grid for YouTube full performances + red See YouTube Channel for More CTA button.</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Resources page is now hidden (direct URL only). Dropdown parent links to # not /resources</t>
+          <t>Resources dropdown parent links to # (not /resources). Page still accessible via direct URL only.</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Fixed desktop layout: reduced font size, added whitespace-nowrap, responsive sizing. Nav now uses lg breakpoint for 8 items</t>
+          <t>Fixed desktop: responsive text-sm/lg:text-base, whitespace-nowrap, nav breakpoint changed md to lg for 8 items.</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Created 3 new sub-pages: /workshops/foundations (3 workshops), /workshops/discipleship (3 workshops), /workshops/advanced (1 workshop). Main workshops page shows 3 tracks with image tiles like Performances page. Generic images for now.</t>
+          <t>3 new sub-pages: /workshops/foundations (3), /workshops/discipleship (3), /workshops/advanced (1). Main page shows 3 tracks with image tiles. Generic images for now.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -847,12 +847,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Homepage - Hero CTA</t>
+          <t>Homepage Hero</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Changed to single Book Jeremy button (was Invite Jeremy + Refer Jeremy)</t>
+          <t>Single Book Jeremy button (replaced Invite Jeremy + Refer Jeremy dual buttons).</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -869,12 +869,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Homepage - Social Proof</t>
+          <t>Homepage Social Proof</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Added endorsement quote section before service tiles with Read More Endorsements link</t>
+          <t>Endorsement quote section added BEFORE service tiles (line 103) with Read More Endorsements link.</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>New 8-item nav: Home | Performances | Workshops | Speaking | Endorsements | Resources (Dropdown) | Events | Book Jeremy (button)</t>
+          <t>New 8-item nav: Home | Performances | Workshops | Speaking | Endorsements | Resources (Dropdown: Store, Videos, Interviews, Blog) | Events | Book Jeremy (button)</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>SEO Issue 4: Approved - NEEDS: Cannot read Google Doc to get details. Kevin please specify what Issue 4 is.</t>
+          <t>SEO Issue 4: Approved but BLOCKED — cannot read Google Doc. Please paste the Issue 4 text.</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>SEO Issue 5: Approved - NEEDS: Cannot read Google Doc to get details. Kevin please specify what Issue 5 is.</t>
+          <t>SEO Issue 5: Approved but BLOCKED — cannot read Google Doc. Please paste the Issue 5 text.</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Homepage - Subtitle</t>
+          <t>Homepage Subtitle</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Added qualifier line: Available for churches, conferences, camps, schools, and special events (below Performances | Workshops | Speaking)</t>
+          <t>Added qualifier: Available for churches, conferences, camps, schools, and special events (below Performances | Workshops | Speaking tagline).</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -971,8 +971,26 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Typography Fix</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Base font reduced 18px to 16px. Global Dancing Script on h1-h4. Body headings (event titles, card titles, category labels) overridden with font-sans. Modal description text-sm.</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D22"/>
+  <autoFilter ref="A1:D23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>